<commit_message>
Switch currency to USD, clarify units, improve month picker UX
- Figures relabeled BRL -> USD thousands across dashboard, PDF and workbook
- Company renamed to Meridian Industries Inc. for an international framing
- Month selector: dropdown to jump + prev/next arrows for one-click stepping
  (replaces the imprecise slider)
</commit_message>
<xml_diff>
--- a/data/raw_pnl.xlsx
+++ b/data/raw_pnl.xlsx
@@ -454,14 +454,14 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>MERIDIAN INDUSTRIES S.A.</t>
+          <t>MERIDIAN INDUSTRIES INC.</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Monthly Management P&amp;L  —  values in BRL '000  —  CONFIDENTIAL</t>
+          <t>Monthly Management P&amp;L  —  figures in USD thousands  —  CONFIDENTIAL</t>
         </is>
       </c>
     </row>
@@ -2218,7 +2218,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Annual Budget (BRL '000)</t>
+          <t>Annual Budget (USD '000)</t>
         </is>
       </c>
     </row>

</xml_diff>